<commit_message>
Move information sources to the Excel
</commit_message>
<xml_diff>
--- a/input/requirements/Condition.xlsx
+++ b/input/requirements/Condition.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahenket/Development/GitHub/Nictiz/GBB-IG/input/requirements/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edelman_nict1\IGs\GBB-IG\input\requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED832230-90A2-B141-8A59-508F66A307AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E15BA777-63BA-4A20-8B94-138FB720C249}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-140" yWindow="-26660" windowWidth="43920" windowHeight="26260" activeTab="1" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
   </bookViews>
   <sheets>
     <sheet name="Uitleg" sheetId="5" r:id="rId1"/>
@@ -50,9 +50,9 @@
   <commentList>
     <comment ref="C5" authorId="0" shapeId="0" xr:uid="{CD16CA43-E215-4DCF-A4C0-2D380EB1C0BC}">
       <text>
-        <t xml:space="preserve">[Opmerkingenthread]
-U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
-Opmerking:
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     Uit Scope en Usage van Condition FHIR R4 v4.0.1 </t>
       </text>
     </comment>
@@ -73,9 +73,9 @@
   <commentList>
     <comment ref="K20" authorId="0" shapeId="0" xr:uid="{B3533A99-0CB6-4646-9417-20A66FEFD573}">
       <text>
-        <t>[Opmerkingenthread]
-U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
-Opmerking:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     1. Actief
 2. Inactief
 Kortere waardelijst</t>
@@ -83,41 +83,41 @@
     </comment>
     <comment ref="K26" authorId="1" shapeId="0" xr:uid="{20B2A504-5F6F-4996-9921-E2104F9548D8}">
       <text>
-        <t>[Opmerkingenthread]
-U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
-Opmerking:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     Wel in metadata!</t>
       </text>
     </comment>
     <comment ref="E29" authorId="2" shapeId="0" xr:uid="{DC3A08E9-01DD-48D1-B7F5-357810DE5428}">
       <text>
-        <t>[Opmerkingenthread]
-U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
-Opmerking:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     Onduidelijk welke waardelijst gehandeerd moet worden</t>
       </text>
     </comment>
     <comment ref="B31" authorId="3" shapeId="0" xr:uid="{035A58F6-6A6B-4788-883F-2110C3BA07ED}">
       <text>
-        <t>[Opmerkingenthread]
-U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
-Opmerking:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     ter discussie</t>
       </text>
     </comment>
     <comment ref="C31" authorId="4" shapeId="0" xr:uid="{00D6E7CD-1959-4C9A-8BC1-A1E323A0102F}">
       <text>
-        <t>[Opmerkingenthread]
-U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
-Opmerking:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     ter discussie</t>
       </text>
     </comment>
     <comment ref="C39" authorId="5" shapeId="0" xr:uid="{065B39A6-9843-49BF-88E8-0C2BF95F8D00}">
       <text>
-        <t>[Opmerkingenthread]
-U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
-Opmerking:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     ter discussie</t>
       </text>
     </comment>
@@ -126,7 +126,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="391">
   <si>
     <t>Veld</t>
   </si>
@@ -1565,6 +1565,15 @@
 - nadereSpecificatieProbleemNaam heeft in ZIBFHIR-145 een mapping gekregen op FHIR, maar is duidelijker in openEHR gemodelleerd als "variant" (echter variant is specifieker, dan LIMS/ZIB wil duiden )
 -specialistcontact: in openEHR is het onduidelijk, mogelijk other participants mits je aan kan geven dat het een voorkeurscontactpersoon is. in FHIR ook niet ideaal, namelijk note.text of via careteam.reason</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">* Logisch informatie model EHDSCondition versie 1.0.0
+* Verplichte elementen uit FHIR R4 Condition 
+* Verplichte elementen uit openEHR Problem / Diagnosis versie 1.7.4 
+* Zib Probleem uit publicatie 2017 
+* Zib Probleem uit publicatie 2020 
+* Informatiestandaard BgZ-MSZ versie 2.0.2 
+* Usecase Spoedsamenvatting van informatiestandaard Acute Zorg versie 2.2.0 </t>
   </si>
 </sst>
 </file>
@@ -1891,7 +1900,7 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="21">
     <dxf>
@@ -1985,46 +1994,6 @@
       </border>
     </dxf>
     <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2090,6 +2059,46 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2811,7 +2820,7 @@
   <autoFilter ref="A2:C13" xr:uid="{7AAA9086-205B-4EC4-8920-A2DD04D02676}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{BDCFF82A-D4BE-440B-90DF-AA26F6831D5C}" name="Veld"/>
-    <tableColumn id="2" xr3:uid="{77503B9E-152C-4B39-87F4-D4FBBF1B3BDA}" name="Uitleg" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{77503B9E-152C-4B39-87F4-D4FBBF1B3BDA}" name="Uitleg" dataDxfId="20"/>
     <tableColumn id="5" xr3:uid="{B530BE2A-715C-42B8-BFE1-95637D35484B}" name="Beschrijving"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2819,36 +2828,36 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1B14A882-8085-4978-86D3-1A5B42023C72}" name="Tabel3" displayName="Tabel3" ref="A1:E17" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1B14A882-8085-4978-86D3-1A5B42023C72}" name="Tabel3" displayName="Tabel3" ref="A1:E17" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
   <autoFilter ref="A1:E17" xr:uid="{1B14A882-8085-4978-86D3-1A5B42023C72}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{2D5F85E5-856C-4A15-8C5D-D8D344B8F13C}" name="Type bron" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{062A7D5A-6D4F-45DD-9A5C-7A2D82A1266A}" name="Naam bron" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{24E64AAE-4BAD-402C-98B7-B46BE371B39E}" name="Toelichting" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{98DE6918-807C-41E0-ACBA-1E2221CF05FC}" name="Informatiebehoefte verwerkt in sheet 'informatiebeheofte'" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{8CFF4D4C-ABDD-49BC-8B49-237193168687}" name="Link naar bron informatie" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{2D5F85E5-856C-4A15-8C5D-D8D344B8F13C}" name="Type bron" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{062A7D5A-6D4F-45DD-9A5C-7A2D82A1266A}" name="Naam bron" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{24E64AAE-4BAD-402C-98B7-B46BE371B39E}" name="Toelichting" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{98DE6918-807C-41E0-ACBA-1E2221CF05FC}" name="Informatiebehoefte verwerkt in sheet 'informatiebeheofte'" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{8CFF4D4C-ABDD-49BC-8B49-237193168687}" name="Link naar bron informatie" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2D02605E-6993-49A7-90CB-92D41480A08E}" name="Tabel6" displayName="Tabel6" ref="A2:N59" totalsRowShown="0" headerRowDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2D02605E-6993-49A7-90CB-92D41480A08E}" name="Tabel6" displayName="Tabel6" ref="A2:N59" totalsRowShown="0" headerRowDxfId="12">
   <autoFilter ref="A2:N59" xr:uid="{2D02605E-6993-49A7-90CB-92D41480A08E}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{51E2B1E8-BF1C-4C85-9A83-8C69A4006993}" name="Nummer" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{021C00E0-4FF4-4652-B8E3-674B1F145954}" name="Naam" dataDxfId="18"/>
+    <tableColumn id="1" xr3:uid="{51E2B1E8-BF1C-4C85-9A83-8C69A4006993}" name="Nummer" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{021C00E0-4FF4-4652-B8E3-674B1F145954}" name="Naam" dataDxfId="10"/>
     <tableColumn id="12" xr3:uid="{721FE94A-B8C9-44E1-A03C-56E48CDCE2A3}" name="data-element"/>
-    <tableColumn id="3" xr3:uid="{12776FCA-6A89-4E9E-907F-2E30F0D43DA3}" name="Omschrijving" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{9E28C4DB-2A8B-484B-80F1-321440976652}" name="Variabiliteit" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{12776FCA-6A89-4E9E-907F-2E30F0D43DA3}" name="Omschrijving" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{9E28C4DB-2A8B-484B-80F1-321440976652}" name="Variabiliteit" dataDxfId="8"/>
     <tableColumn id="5" xr3:uid="{6FA3E114-7382-4230-B15E-A8DB28B8CE4B}" name="Aanwezigheid"/>
     <tableColumn id="6" xr3:uid="{E8FFDBDF-8B88-4089-89D0-252402D12764}" name="Verleden/heden/toekomst"/>
     <tableColumn id="7" xr3:uid="{BB9C62AB-9839-431A-90A2-B6A6D70DF1FB}" name="Herkomst"/>
     <tableColumn id="8" xr3:uid="{6BE87E7D-EFAE-42FD-9334-11E5EBAC9DC3}" name="Komt het in FHIR R4 voor?"/>
     <tableColumn id="9" xr3:uid="{C6EE00AA-2B37-4BE3-B349-AF61C6E68575}" name="Komt het in openEHR voor?"/>
     <tableColumn id="10" xr3:uid="{943D4BF3-315C-41FB-99E4-8DB8C54604A4}" name="Komt voor in ZIBProbleem-v4.4? (2020)"/>
-    <tableColumn id="14" xr3:uid="{8B1A7EB4-D690-4A36-9698-ACA592C2A715}" name="Komt voor in ZIBProbleem? (2017)" dataDxfId="15"/>
-    <tableColumn id="13" xr3:uid="{51A57E0A-A216-45BB-973D-E0D8C72BEEEC}" name="Komt voor in ZIBProbleem? (2024)" dataDxfId="14"/>
+    <tableColumn id="14" xr3:uid="{8B1A7EB4-D690-4A36-9698-ACA592C2A715}" name="Komt voor in ZIBProbleem? (2017)" dataDxfId="7"/>
+    <tableColumn id="13" xr3:uid="{51A57E0A-A216-45BB-973D-E0D8C72BEEEC}" name="Komt voor in ZIBProbleem? (2024)" dataDxfId="6"/>
     <tableColumn id="11" xr3:uid="{E7EDB106-7E3F-4122-A864-3B3AE59C9D87}" name="Opmerking"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3230,15 +3239,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F1013F7-63B2-4F83-92B0-1C8153859891}">
   <dimension ref="A1:C19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="218.5" customWidth="1"/>
+    <col min="1" max="1" width="218.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3"/>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B18">
         <f>(510*132.5) + (160*132.5)</f>
         <v>88775</v>
@@ -3247,7 +3256,7 @@
         <v>5832</v>
       </c>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B19">
         <f>(542*132.5)</f>
         <v>71815</v>
@@ -3265,17 +3274,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC1E3B3-D087-4A2B-920B-9BA971FAD64B}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="46.6640625" customWidth="1"/>
-    <col min="3" max="3" width="59.6640625" customWidth="1"/>
+    <col min="2" max="2" width="46.7109375" customWidth="1"/>
+    <col min="3" max="3" width="59.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="3"/>
     </row>
-    <row r="2" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -3286,7 +3295,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -3297,7 +3306,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="96" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -3308,7 +3317,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="304" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="330" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -3319,7 +3328,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="64" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -3330,7 +3339,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -3341,7 +3350,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -3352,7 +3361,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="96" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" ht="105" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -3363,18 +3372,18 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" ht="135" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>23</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+      <c r="C10" s="4" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -3385,7 +3394,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="256" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" ht="315" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -3394,7 +3403,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>30</v>
       </c>
@@ -3416,16 +3425,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8AA88E1-0CFC-4A69-A682-35DA329C9688}">
   <dimension ref="A1:E17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.33203125" customWidth="1"/>
-    <col min="2" max="2" width="51.33203125" customWidth="1"/>
-    <col min="3" max="3" width="67.33203125" customWidth="1"/>
+    <col min="1" max="1" width="19.28515625" customWidth="1"/>
+    <col min="2" max="2" width="51.28515625" customWidth="1"/>
+    <col min="3" max="3" width="67.28515625" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="5" width="58.1640625" customWidth="1"/>
+    <col min="5" max="5" width="58.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>31</v>
       </c>
@@ -3442,7 +3451,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="48" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>36</v>
       </c>
@@ -3459,7 +3468,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>36</v>
       </c>
@@ -3476,7 +3485,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>36</v>
       </c>
@@ -3493,7 +3502,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>46</v>
       </c>
@@ -3508,7 +3517,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>46</v>
       </c>
@@ -3523,7 +3532,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>46</v>
       </c>
@@ -3538,7 +3547,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="48" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>55</v>
       </c>
@@ -3555,7 +3564,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="48" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>55</v>
       </c>
@@ -3572,7 +3581,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>55</v>
       </c>
@@ -3581,49 +3590,49 @@
       <c r="D10" s="3"/>
       <c r="E10" s="6"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="6"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="6"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="4"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
       <c r="E14" s="4"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="4"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
       <c r="E16" s="4"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -3650,25 +3659,25 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7034CDAF-2A08-4BE8-92C3-F4E7A6F24E1B}">
   <dimension ref="A1:O65"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.5" customWidth="1"/>
-    <col min="2" max="2" width="29.33203125" customWidth="1"/>
-    <col min="3" max="3" width="32.6640625" customWidth="1"/>
-    <col min="4" max="4" width="87.5" style="3" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="29.28515625" customWidth="1"/>
+    <col min="3" max="3" width="32.7109375" customWidth="1"/>
+    <col min="4" max="4" width="87.42578125" style="3" customWidth="1"/>
     <col min="5" max="5" width="78" style="3" customWidth="1"/>
-    <col min="6" max="6" width="18.6640625" customWidth="1"/>
-    <col min="7" max="7" width="11.5" customWidth="1"/>
-    <col min="8" max="8" width="32.5" customWidth="1"/>
-    <col min="9" max="9" width="28.1640625" customWidth="1"/>
-    <col min="10" max="10" width="51.33203125" customWidth="1"/>
-    <col min="11" max="11" width="38.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="38.5" customWidth="1"/>
-    <col min="14" max="14" width="33.33203125" customWidth="1"/>
+    <col min="6" max="6" width="18.7109375" customWidth="1"/>
+    <col min="7" max="7" width="11.42578125" customWidth="1"/>
+    <col min="8" max="8" width="32.42578125" customWidth="1"/>
+    <col min="9" max="9" width="28.140625" customWidth="1"/>
+    <col min="10" max="10" width="51.28515625" customWidth="1"/>
+    <col min="11" max="11" width="38.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="38.42578125" customWidth="1"/>
+    <col min="14" max="14" width="33.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="99.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" ht="99.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>62</v>
       </c>
@@ -3712,7 +3721,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="182.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" ht="182.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="19" t="s">
         <v>80</v>
       </c>
@@ -3743,7 +3752,7 @@
       <c r="N3" s="19"/>
       <c r="O3" s="9"/>
     </row>
-    <row r="4" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>85</v>
       </c>
@@ -3770,7 +3779,7 @@
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
     </row>
-    <row r="5" spans="1:15" ht="48" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
         <v>91</v>
       </c>
@@ -3798,7 +3807,7 @@
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
     </row>
-    <row r="6" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>96</v>
       </c>
@@ -3826,7 +3835,7 @@
       <c r="M6" s="3"/>
       <c r="N6" s="3"/>
     </row>
-    <row r="7" spans="1:15" ht="80" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" ht="105" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>99</v>
       </c>
@@ -3854,7 +3863,7 @@
       <c r="M7" s="3"/>
       <c r="N7" s="3"/>
     </row>
-    <row r="8" spans="1:15" ht="32" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>103</v>
       </c>
@@ -3875,7 +3884,7 @@
       <c r="M8" s="3"/>
       <c r="N8" s="3"/>
     </row>
-    <row r="9" spans="1:15" ht="48" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>106</v>
       </c>
@@ -3907,7 +3916,7 @@
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
     </row>
-    <row r="10" spans="1:15" ht="32" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>114</v>
       </c>
@@ -3934,7 +3943,7 @@
       <c r="M10" s="3"/>
       <c r="N10" s="3"/>
     </row>
-    <row r="11" spans="1:15" ht="64" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15" ht="75" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
         <v>119</v>
       </c>
@@ -3967,7 +3976,7 @@
       <c r="M11" s="3"/>
       <c r="N11" s="3"/>
     </row>
-    <row r="12" spans="1:15" ht="96" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15" ht="105" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
         <v>127</v>
       </c>
@@ -4003,7 +4012,7 @@
       <c r="M12" s="3"/>
       <c r="N12" s="3"/>
     </row>
-    <row r="13" spans="1:15" ht="180.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15" ht="180.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>135</v>
       </c>
@@ -4039,7 +4048,7 @@
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
     </row>
-    <row r="14" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
         <v>142</v>
       </c>
@@ -4073,7 +4082,7 @@
       <c r="M14" s="3"/>
       <c r="N14" s="3"/>
     </row>
-    <row r="15" spans="1:15" ht="135" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15" ht="135" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>147</v>
       </c>
@@ -4107,7 +4116,7 @@
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
     </row>
-    <row r="16" spans="1:15" ht="16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
         <v>154</v>
       </c>
@@ -4125,7 +4134,7 @@
       <c r="M16" s="3"/>
       <c r="N16" s="3"/>
     </row>
-    <row r="17" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
         <v>156</v>
       </c>
@@ -4159,7 +4168,7 @@
       <c r="M17" s="3"/>
       <c r="N17" s="3"/>
     </row>
-    <row r="18" spans="1:14" ht="70.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:14" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
         <v>163</v>
       </c>
@@ -4187,7 +4196,7 @@
       <c r="M18" s="3"/>
       <c r="N18" s="3"/>
     </row>
-    <row r="19" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>168</v>
       </c>
@@ -4208,7 +4217,7 @@
       <c r="M19" s="3"/>
       <c r="N19" s="3"/>
     </row>
-    <row r="20" spans="1:14" ht="101.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:14" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
         <v>171</v>
       </c>
@@ -4246,7 +4255,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="108" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:14" ht="108" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
         <v>179</v>
       </c>
@@ -4277,7 +4286,7 @@
       <c r="M21" s="3"/>
       <c r="N21" s="3"/>
     </row>
-    <row r="22" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="19" t="s">
         <v>183</v>
       </c>
@@ -4295,7 +4304,7 @@
       <c r="M22" s="3"/>
       <c r="N22" s="3"/>
     </row>
-    <row r="23" spans="1:14" ht="64" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
         <v>185</v>
       </c>
@@ -4335,7 +4344,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="80" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:14" ht="75" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
         <v>195</v>
       </c>
@@ -4363,7 +4372,7 @@
       <c r="M24" s="3"/>
       <c r="N24" s="5"/>
     </row>
-    <row r="25" spans="1:14" ht="149.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:14" ht="149.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
         <v>199</v>
       </c>
@@ -4391,7 +4400,7 @@
       <c r="M25" s="3"/>
       <c r="N25" s="3"/>
     </row>
-    <row r="26" spans="1:14" ht="48" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
         <v>204</v>
       </c>
@@ -4425,7 +4434,7 @@
       <c r="M26" s="3"/>
       <c r="N26" s="3"/>
     </row>
-    <row r="27" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
         <v>210</v>
       </c>
@@ -4449,7 +4458,7 @@
       <c r="M27" s="3"/>
       <c r="N27" s="3"/>
     </row>
-    <row r="28" spans="1:14" ht="47.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:14" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
         <v>215</v>
       </c>
@@ -4473,7 +4482,7 @@
       <c r="I28" s="3"/>
       <c r="N28" s="3"/>
     </row>
-    <row r="29" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="19" t="s">
         <v>219</v>
       </c>
@@ -4501,7 +4510,7 @@
       <c r="M29" s="3"/>
       <c r="N29" s="3"/>
     </row>
-    <row r="30" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
         <v>223</v>
       </c>
@@ -4529,7 +4538,7 @@
       <c r="M30" s="3"/>
       <c r="N30" s="3"/>
     </row>
-    <row r="31" spans="1:14" ht="219" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:14" ht="219" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
         <v>228</v>
       </c>
@@ -4557,7 +4566,7 @@
       <c r="M31" s="3"/>
       <c r="N31" s="3"/>
     </row>
-    <row r="32" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
         <v>233</v>
       </c>
@@ -4586,7 +4595,7 @@
       <c r="M32" s="3"/>
       <c r="N32" s="3"/>
     </row>
-    <row r="33" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
         <v>240</v>
       </c>
@@ -4609,7 +4618,7 @@
       </c>
       <c r="N33" s="3"/>
     </row>
-    <row r="34" spans="1:14" ht="162" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:14" ht="162" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="19" t="s">
         <v>243</v>
       </c>
@@ -4637,7 +4646,7 @@
       <c r="M34" s="3"/>
       <c r="N34" s="3"/>
     </row>
-    <row r="35" spans="1:14" ht="121.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:14" ht="121.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="9" t="s">
         <v>248</v>
       </c>
@@ -4665,7 +4674,7 @@
       <c r="M35" s="3"/>
       <c r="N35" s="3"/>
     </row>
-    <row r="36" spans="1:14" ht="32" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
         <v>253</v>
       </c>
@@ -4692,7 +4701,7 @@
       <c r="M36" s="3"/>
       <c r="N36" s="3"/>
     </row>
-    <row r="37" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="19" t="s">
         <v>259</v>
       </c>
@@ -4720,7 +4729,7 @@
       <c r="M37" s="3"/>
       <c r="N37" s="3"/>
     </row>
-    <row r="38" spans="1:14" ht="66.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:14" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="19" t="s">
         <v>263</v>
       </c>
@@ -4748,7 +4757,7 @@
       <c r="M38" s="3"/>
       <c r="N38" s="3"/>
     </row>
-    <row r="39" spans="1:14" ht="178.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:14" ht="178.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="9" t="s">
         <v>267</v>
       </c>
@@ -4776,7 +4785,7 @@
       <c r="M39" s="3"/>
       <c r="N39" s="3"/>
     </row>
-    <row r="40" spans="1:14" ht="135" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:14" ht="135" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="19" t="s">
         <v>271</v>
       </c>
@@ -4808,7 +4817,7 @@
       <c r="M40" s="3"/>
       <c r="N40" s="3"/>
     </row>
-    <row r="41" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="9" t="s">
         <v>276</v>
       </c>
@@ -4836,7 +4845,7 @@
       <c r="M41" s="3"/>
       <c r="N41" s="3"/>
     </row>
-    <row r="42" spans="1:14" ht="98.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:14" ht="98.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="9" t="s">
         <v>280</v>
       </c>
@@ -4864,7 +4873,7 @@
       <c r="M42" s="3"/>
       <c r="N42" s="3"/>
     </row>
-    <row r="43" spans="1:14" ht="32" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="19" t="s">
         <v>285</v>
       </c>
@@ -4896,7 +4905,7 @@
       <c r="M43" s="3"/>
       <c r="N43" s="3"/>
     </row>
-    <row r="44" spans="1:14" ht="48" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A44" s="9"/>
       <c r="B44" s="3"/>
       <c r="C44" s="10"/>
@@ -4913,7 +4922,7 @@
       <c r="M44" s="3"/>
       <c r="N44" s="3"/>
     </row>
-    <row r="45" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="19" t="s">
         <v>292</v>
       </c>
@@ -4947,7 +4956,7 @@
       <c r="M45" s="3"/>
       <c r="N45" s="3"/>
     </row>
-    <row r="46" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="9" t="s">
         <v>299</v>
       </c>
@@ -4966,7 +4975,7 @@
       <c r="M46" s="3"/>
       <c r="N46" s="3"/>
     </row>
-    <row r="47" spans="1:14" ht="59.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:14" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="9" t="s">
         <v>301</v>
       </c>
@@ -4994,7 +5003,7 @@
       <c r="M47" s="3"/>
       <c r="N47" s="3"/>
     </row>
-    <row r="48" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" s="19" t="s">
         <v>305</v>
       </c>
@@ -5026,7 +5035,7 @@
       <c r="M48" s="3"/>
       <c r="N48" s="3"/>
     </row>
-    <row r="49" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="19" t="s">
         <v>311</v>
       </c>
@@ -5051,7 +5060,7 @@
       <c r="M49" s="3"/>
       <c r="N49" s="3"/>
     </row>
-    <row r="50" spans="1:14" ht="32" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="19" t="s">
         <v>314</v>
       </c>
@@ -5076,7 +5085,7 @@
       <c r="M50" s="3"/>
       <c r="N50" s="3"/>
     </row>
-    <row r="51" spans="1:14" ht="32" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="19" t="s">
         <v>317</v>
       </c>
@@ -5110,7 +5119,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="52" spans="1:14" ht="32" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="9"/>
       <c r="B52" s="3"/>
       <c r="C52" s="10"/>
@@ -5127,7 +5136,7 @@
       <c r="M52" s="3"/>
       <c r="N52" s="4"/>
     </row>
-    <row r="53" spans="1:14" ht="32" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="9" t="s">
         <v>325</v>
       </c>
@@ -5145,7 +5154,7 @@
       <c r="M53" s="3"/>
       <c r="N53" s="3"/>
     </row>
-    <row r="54" spans="1:14" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:14" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="19" t="s">
         <v>327</v>
       </c>
@@ -5179,7 +5188,7 @@
       <c r="M54" s="25"/>
       <c r="N54" s="3"/>
     </row>
-    <row r="55" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="9" t="s">
         <v>334</v>
       </c>
@@ -5207,7 +5216,7 @@
       <c r="M55" s="17"/>
       <c r="N55" s="3"/>
     </row>
-    <row r="56" spans="1:14" ht="32" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A56" s="19" t="s">
         <v>338</v>
       </c>
@@ -5239,7 +5248,7 @@
       <c r="M56" s="3"/>
       <c r="N56" s="3"/>
     </row>
-    <row r="57" spans="1:14" ht="32" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A57" s="19" t="s">
         <v>344</v>
       </c>
@@ -5271,7 +5280,7 @@
       <c r="M57" s="3"/>
       <c r="N57" s="3"/>
     </row>
-    <row r="58" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="19" t="s">
         <v>351</v>
       </c>
@@ -5303,7 +5312,7 @@
       <c r="M58" s="3"/>
       <c r="N58" s="3"/>
     </row>
-    <row r="59" spans="1:14" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:14" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="9" t="s">
         <v>355</v>
       </c>
@@ -5326,15 +5335,15 @@
         <v>361</v>
       </c>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B63" s="28"/>
       <c r="C63" s="28"/>
     </row>
-    <row r="64" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B64" s="29"/>
       <c r="C64" s="30"/>
     </row>
-    <row r="65" spans="2:3" ht="16" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="2:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B65" s="28"/>
       <c r="C65" s="28"/>
     </row>
@@ -5358,17 +5367,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{273AFAA3-99F7-4E93-9580-DCAE2B14D938}">
   <dimension ref="A1:G2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.1640625" customWidth="1"/>
-    <col min="2" max="2" width="18.5" customWidth="1"/>
-    <col min="4" max="4" width="15.1640625" customWidth="1"/>
-    <col min="5" max="5" width="16.6640625" customWidth="1"/>
-    <col min="6" max="6" width="16.5" customWidth="1"/>
-    <col min="7" max="7" width="41.5" customWidth="1"/>
+    <col min="1" max="1" width="19.140625" customWidth="1"/>
+    <col min="2" max="2" width="18.42578125" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" customWidth="1"/>
+    <col min="7" max="7" width="41.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="195.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="195.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>362</v>
       </c>
@@ -5391,7 +5400,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>364</v>
       </c>
@@ -5423,10 +5432,10 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2489EBC-5098-4697-9724-F190D24E1C3D}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="111" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1" ht="111" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>367</v>
       </c>
@@ -5440,13 +5449,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0062C35-A590-498D-8635-16DE3DC0B82A}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.5" customWidth="1"/>
+    <col min="1" max="1" width="36.42578125" customWidth="1"/>
     <col min="2" max="2" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>100</v>
       </c>
@@ -5454,7 +5463,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>368</v>
       </c>
@@ -5462,7 +5471,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>370</v>
       </c>
@@ -5478,15 +5487,15 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9E8E4E8-143C-4C64-99FB-1306F2338EFB}">
   <dimension ref="A2:J9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="27.6640625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="27.5" style="3" customWidth="1"/>
-    <col min="4" max="4" width="60.1640625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="47.6640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="27.7109375" style="3" customWidth="1"/>
+    <col min="3" max="3" width="27.42578125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="60.140625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="47.7109375" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B2" s="15" t="s">
         <v>371</v>
       </c>
@@ -5494,7 +5503,7 @@
       <c r="D2" s="12"/>
       <c r="E2" s="12"/>
     </row>
-    <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B3" s="16" t="s">
         <v>372</v>
       </c>
@@ -5508,7 +5517,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="156" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" ht="156" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="14" t="s">
         <v>375</v>
       </c>
@@ -5520,7 +5529,7 @@
       </c>
       <c r="E4" s="14"/>
     </row>
-    <row r="5" spans="1:10" ht="182.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" ht="182.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="14" t="s">
         <v>378</v>
       </c>
@@ -5532,7 +5541,7 @@
       </c>
       <c r="E5" s="14"/>
     </row>
-    <row r="6" spans="1:10" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19"/>
       <c r="B6" s="3" t="s">
         <v>339</v>
@@ -5549,7 +5558,7 @@
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
     </row>
-    <row r="7" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B7" s="14" t="s">
         <v>382</v>
       </c>
@@ -5561,7 +5570,7 @@
       </c>
       <c r="E7" s="14"/>
     </row>
-    <row r="8" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B8" s="14" t="s">
         <v>384</v>
       </c>
@@ -5573,7 +5582,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="80" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" ht="90" x14ac:dyDescent="0.25">
       <c r="B9" s="14"/>
       <c r="C9" s="14" t="s">
         <v>387</v>
@@ -5592,6 +5601,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
@@ -5600,15 +5618,6 @@
     <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5819,6 +5828,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -5831,14 +5848,6 @@
     <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Condition: Update requirements test
</commit_message>
<xml_diff>
--- a/input/requirements/Condition.xlsx
+++ b/input/requirements/Condition.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edelman_nict1\IGs\GBB-IG\input\requirements\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/onnogieling/dev/GBB-IG/input/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E15BA777-63BA-4A20-8B94-138FB720C249}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ACC6E45-F058-3147-A954-25D8F093EA11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
   </bookViews>
   <sheets>
     <sheet name="Uitleg" sheetId="5" r:id="rId1"/>
@@ -3239,15 +3239,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F1013F7-63B2-4F83-92B0-1C8153859891}">
   <dimension ref="A1:C19"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="218.42578125" customWidth="1"/>
+    <col min="1" max="1" width="218.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3"/>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B18">
         <f>(510*132.5) + (160*132.5)</f>
         <v>88775</v>
@@ -3256,7 +3256,7 @@
         <v>5832</v>
       </c>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B19">
         <f>(542*132.5)</f>
         <v>71815</v>
@@ -3274,17 +3274,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC1E3B3-D087-4A2B-920B-9BA971FAD64B}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="46.7109375" customWidth="1"/>
-    <col min="3" max="3" width="59.7109375" customWidth="1"/>
+    <col min="2" max="2" width="46.6640625" customWidth="1"/>
+    <col min="3" max="3" width="59.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="3"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -3295,7 +3295,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -3306,7 +3306,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="105" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="96" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -3317,7 +3317,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="330" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="304" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -3328,7 +3328,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="64" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -3339,7 +3339,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="48" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -3350,7 +3350,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="48" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -3361,7 +3361,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="105" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="96" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -3372,7 +3372,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="135" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="128" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -3383,7 +3383,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="48" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -3394,7 +3394,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="315" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="256" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -3403,7 +3403,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>30</v>
       </c>
@@ -3425,16 +3425,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8AA88E1-0CFC-4A69-A682-35DA329C9688}">
   <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" customWidth="1"/>
-    <col min="2" max="2" width="51.28515625" customWidth="1"/>
-    <col min="3" max="3" width="67.28515625" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" customWidth="1"/>
+    <col min="2" max="2" width="51.33203125" customWidth="1"/>
+    <col min="3" max="3" width="67.33203125" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="5" width="58.140625" customWidth="1"/>
+    <col min="5" max="5" width="58.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>31</v>
       </c>
@@ -3451,7 +3451,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="48" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>36</v>
       </c>
@@ -3468,7 +3468,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>36</v>
       </c>
@@ -3485,7 +3485,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>36</v>
       </c>
@@ -3502,7 +3502,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>46</v>
       </c>
@@ -3517,7 +3517,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>46</v>
       </c>
@@ -3532,7 +3532,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>46</v>
       </c>
@@ -3547,7 +3547,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="48" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>55</v>
       </c>
@@ -3564,7 +3564,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="48" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>55</v>
       </c>
@@ -3581,7 +3581,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>55</v>
       </c>
@@ -3590,49 +3590,49 @@
       <c r="D10" s="3"/>
       <c r="E10" s="6"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="6"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="6"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="4"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
       <c r="E14" s="4"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="4"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
       <c r="E16" s="4"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -3659,25 +3659,25 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7034CDAF-2A08-4BE8-92C3-F4E7A6F24E1B}">
   <dimension ref="A1:O65"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" customWidth="1"/>
-    <col min="2" max="2" width="29.28515625" customWidth="1"/>
-    <col min="3" max="3" width="32.7109375" customWidth="1"/>
-    <col min="4" max="4" width="87.42578125" style="3" customWidth="1"/>
+    <col min="1" max="1" width="11.5" customWidth="1"/>
+    <col min="2" max="2" width="29.33203125" customWidth="1"/>
+    <col min="3" max="3" width="32.6640625" customWidth="1"/>
+    <col min="4" max="4" width="87.5" style="3" customWidth="1"/>
     <col min="5" max="5" width="78" style="3" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="11.42578125" customWidth="1"/>
-    <col min="8" max="8" width="32.42578125" customWidth="1"/>
-    <col min="9" max="9" width="28.140625" customWidth="1"/>
-    <col min="10" max="10" width="51.28515625" customWidth="1"/>
-    <col min="11" max="11" width="38.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="38.42578125" customWidth="1"/>
-    <col min="14" max="14" width="33.28515625" customWidth="1"/>
+    <col min="6" max="6" width="18.6640625" customWidth="1"/>
+    <col min="7" max="7" width="11.5" customWidth="1"/>
+    <col min="8" max="8" width="32.5" customWidth="1"/>
+    <col min="9" max="9" width="28.1640625" customWidth="1"/>
+    <col min="10" max="10" width="51.33203125" customWidth="1"/>
+    <col min="11" max="11" width="38.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="38.5" customWidth="1"/>
+    <col min="14" max="14" width="33.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="99.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" ht="99.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>62</v>
       </c>
@@ -3721,7 +3721,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="182.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" ht="182.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="19" t="s">
         <v>80</v>
       </c>
@@ -3752,11 +3752,11 @@
       <c r="N3" s="19"/>
       <c r="O3" s="9"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="B4" s="8" t="s">
         <v>86</v>
       </c>
       <c r="D4" s="3" t="s">
@@ -3779,12 +3779,11 @@
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
     </row>
-    <row r="5" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" ht="48" x14ac:dyDescent="0.2">
       <c r="A5" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8" t="s">
+      <c r="B5" s="8" t="s">
         <v>92</v>
       </c>
       <c r="D5" s="3" t="s">
@@ -3807,12 +3806,11 @@
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
     </row>
-    <row r="6" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8" t="s">
+      <c r="B6" s="8" t="s">
         <v>86</v>
       </c>
       <c r="D6" s="3" t="s">
@@ -3835,12 +3833,11 @@
       <c r="M6" s="3"/>
       <c r="N6" s="3"/>
     </row>
-    <row r="7" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" ht="80" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8" t="s">
+      <c r="B7" s="8" t="s">
         <v>100</v>
       </c>
       <c r="D7" s="3" t="s">
@@ -3863,7 +3860,7 @@
       <c r="M7" s="3"/>
       <c r="N7" s="3"/>
     </row>
-    <row r="8" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
         <v>103</v>
       </c>
@@ -3884,7 +3881,7 @@
       <c r="M8" s="3"/>
       <c r="N8" s="3"/>
     </row>
-    <row r="9" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" ht="48" x14ac:dyDescent="0.2">
       <c r="A9" s="19" t="s">
         <v>106</v>
       </c>
@@ -3916,7 +3913,7 @@
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
     </row>
-    <row r="10" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="19" t="s">
         <v>114</v>
       </c>
@@ -3943,7 +3940,7 @@
       <c r="M10" s="3"/>
       <c r="N10" s="3"/>
     </row>
-    <row r="11" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" ht="64" x14ac:dyDescent="0.2">
       <c r="A11" s="19" t="s">
         <v>119</v>
       </c>
@@ -3976,7 +3973,7 @@
       <c r="M11" s="3"/>
       <c r="N11" s="3"/>
     </row>
-    <row r="12" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" ht="96" x14ac:dyDescent="0.2">
       <c r="A12" s="19" t="s">
         <v>127</v>
       </c>
@@ -4012,7 +4009,7 @@
       <c r="M12" s="3"/>
       <c r="N12" s="3"/>
     </row>
-    <row r="13" spans="1:15" ht="180.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" ht="180.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="19" t="s">
         <v>135</v>
       </c>
@@ -4048,7 +4045,7 @@
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="19" t="s">
         <v>142</v>
       </c>
@@ -4082,7 +4079,7 @@
       <c r="M14" s="3"/>
       <c r="N14" s="3"/>
     </row>
-    <row r="15" spans="1:15" ht="135" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" ht="135" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
         <v>147</v>
       </c>
@@ -4116,7 +4113,7 @@
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
     </row>
-    <row r="16" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
         <v>154</v>
       </c>
@@ -4134,7 +4131,7 @@
       <c r="M16" s="3"/>
       <c r="N16" s="3"/>
     </row>
-    <row r="17" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="19" t="s">
         <v>156</v>
       </c>
@@ -4168,7 +4165,7 @@
       <c r="M17" s="3"/>
       <c r="N17" s="3"/>
     </row>
-    <row r="18" spans="1:14" ht="70.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" ht="70.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="19" t="s">
         <v>163</v>
       </c>
@@ -4196,7 +4193,7 @@
       <c r="M18" s="3"/>
       <c r="N18" s="3"/>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="9" t="s">
         <v>168</v>
       </c>
@@ -4217,7 +4214,7 @@
       <c r="M19" s="3"/>
       <c r="N19" s="3"/>
     </row>
-    <row r="20" spans="1:14" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" ht="101.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="19" t="s">
         <v>171</v>
       </c>
@@ -4255,7 +4252,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="108" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" ht="108" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="19" t="s">
         <v>179</v>
       </c>
@@ -4286,7 +4283,7 @@
       <c r="M21" s="3"/>
       <c r="N21" s="3"/>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="19" t="s">
         <v>183</v>
       </c>
@@ -4304,7 +4301,7 @@
       <c r="M22" s="3"/>
       <c r="N22" s="3"/>
     </row>
-    <row r="23" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" ht="64" x14ac:dyDescent="0.2">
       <c r="A23" s="9" t="s">
         <v>185</v>
       </c>
@@ -4344,7 +4341,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" ht="80" x14ac:dyDescent="0.2">
       <c r="A24" s="9" t="s">
         <v>195</v>
       </c>
@@ -4372,7 +4369,7 @@
       <c r="M24" s="3"/>
       <c r="N24" s="5"/>
     </row>
-    <row r="25" spans="1:14" ht="149.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" ht="149.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="9" t="s">
         <v>199</v>
       </c>
@@ -4400,7 +4397,7 @@
       <c r="M25" s="3"/>
       <c r="N25" s="3"/>
     </row>
-    <row r="26" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" ht="48" x14ac:dyDescent="0.2">
       <c r="A26" s="19" t="s">
         <v>204</v>
       </c>
@@ -4434,7 +4431,7 @@
       <c r="M26" s="3"/>
       <c r="N26" s="3"/>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="19" t="s">
         <v>210</v>
       </c>
@@ -4458,7 +4455,7 @@
       <c r="M27" s="3"/>
       <c r="N27" s="3"/>
     </row>
-    <row r="28" spans="1:14" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" ht="47.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="19" t="s">
         <v>215</v>
       </c>
@@ -4482,7 +4479,7 @@
       <c r="I28" s="3"/>
       <c r="N28" s="3"/>
     </row>
-    <row r="29" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="19" t="s">
         <v>219</v>
       </c>
@@ -4510,7 +4507,7 @@
       <c r="M29" s="3"/>
       <c r="N29" s="3"/>
     </row>
-    <row r="30" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="19" t="s">
         <v>223</v>
       </c>
@@ -4538,7 +4535,7 @@
       <c r="M30" s="3"/>
       <c r="N30" s="3"/>
     </row>
-    <row r="31" spans="1:14" ht="219" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" ht="219" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="19" t="s">
         <v>228</v>
       </c>
@@ -4566,7 +4563,7 @@
       <c r="M31" s="3"/>
       <c r="N31" s="3"/>
     </row>
-    <row r="32" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="9" t="s">
         <v>233</v>
       </c>
@@ -4595,7 +4592,7 @@
       <c r="M32" s="3"/>
       <c r="N32" s="3"/>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="19" t="s">
         <v>240</v>
       </c>
@@ -4618,7 +4615,7 @@
       </c>
       <c r="N33" s="3"/>
     </row>
-    <row r="34" spans="1:14" ht="162" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" ht="162" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="19" t="s">
         <v>243</v>
       </c>
@@ -4646,7 +4643,7 @@
       <c r="M34" s="3"/>
       <c r="N34" s="3"/>
     </row>
-    <row r="35" spans="1:14" ht="121.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" ht="121.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="9" t="s">
         <v>248</v>
       </c>
@@ -4674,7 +4671,7 @@
       <c r="M35" s="3"/>
       <c r="N35" s="3"/>
     </row>
-    <row r="36" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A36" s="9" t="s">
         <v>253</v>
       </c>
@@ -4701,7 +4698,7 @@
       <c r="M36" s="3"/>
       <c r="N36" s="3"/>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="19" t="s">
         <v>259</v>
       </c>
@@ -4729,7 +4726,7 @@
       <c r="M37" s="3"/>
       <c r="N37" s="3"/>
     </row>
-    <row r="38" spans="1:14" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" ht="66.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="19" t="s">
         <v>263</v>
       </c>
@@ -4757,7 +4754,7 @@
       <c r="M38" s="3"/>
       <c r="N38" s="3"/>
     </row>
-    <row r="39" spans="1:14" ht="178.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" ht="178.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="9" t="s">
         <v>267</v>
       </c>
@@ -4785,7 +4782,7 @@
       <c r="M39" s="3"/>
       <c r="N39" s="3"/>
     </row>
-    <row r="40" spans="1:14" ht="135" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" ht="135" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="19" t="s">
         <v>271</v>
       </c>
@@ -4817,7 +4814,7 @@
       <c r="M40" s="3"/>
       <c r="N40" s="3"/>
     </row>
-    <row r="41" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="9" t="s">
         <v>276</v>
       </c>
@@ -4845,7 +4842,7 @@
       <c r="M41" s="3"/>
       <c r="N41" s="3"/>
     </row>
-    <row r="42" spans="1:14" ht="98.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14" ht="98.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="9" t="s">
         <v>280</v>
       </c>
@@ -4873,7 +4870,7 @@
       <c r="M42" s="3"/>
       <c r="N42" s="3"/>
     </row>
-    <row r="43" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A43" s="19" t="s">
         <v>285</v>
       </c>
@@ -4905,7 +4902,7 @@
       <c r="M43" s="3"/>
       <c r="N43" s="3"/>
     </row>
-    <row r="44" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14" ht="48" x14ac:dyDescent="0.2">
       <c r="A44" s="9"/>
       <c r="B44" s="3"/>
       <c r="C44" s="10"/>
@@ -4922,7 +4919,7 @@
       <c r="M44" s="3"/>
       <c r="N44" s="3"/>
     </row>
-    <row r="45" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="19" t="s">
         <v>292</v>
       </c>
@@ -4956,7 +4953,7 @@
       <c r="M45" s="3"/>
       <c r="N45" s="3"/>
     </row>
-    <row r="46" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" ht="54.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="9" t="s">
         <v>299</v>
       </c>
@@ -4975,7 +4972,7 @@
       <c r="M46" s="3"/>
       <c r="N46" s="3"/>
     </row>
-    <row r="47" spans="1:14" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" ht="59.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="9" t="s">
         <v>301</v>
       </c>
@@ -5003,7 +5000,7 @@
       <c r="M47" s="3"/>
       <c r="N47" s="3"/>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" s="19" t="s">
         <v>305</v>
       </c>
@@ -5035,7 +5032,7 @@
       <c r="M48" s="3"/>
       <c r="N48" s="3"/>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" s="19" t="s">
         <v>311</v>
       </c>
@@ -5060,7 +5057,7 @@
       <c r="M49" s="3"/>
       <c r="N49" s="3"/>
     </row>
-    <row r="50" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A50" s="19" t="s">
         <v>314</v>
       </c>
@@ -5085,7 +5082,7 @@
       <c r="M50" s="3"/>
       <c r="N50" s="3"/>
     </row>
-    <row r="51" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A51" s="19" t="s">
         <v>317</v>
       </c>
@@ -5119,7 +5116,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="52" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A52" s="9"/>
       <c r="B52" s="3"/>
       <c r="C52" s="10"/>
@@ -5136,7 +5133,7 @@
       <c r="M52" s="3"/>
       <c r="N52" s="4"/>
     </row>
-    <row r="53" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A53" s="9" t="s">
         <v>325</v>
       </c>
@@ -5154,7 +5151,7 @@
       <c r="M53" s="3"/>
       <c r="N53" s="3"/>
     </row>
-    <row r="54" spans="1:14" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="19" t="s">
         <v>327</v>
       </c>
@@ -5188,7 +5185,7 @@
       <c r="M54" s="25"/>
       <c r="N54" s="3"/>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A55" s="9" t="s">
         <v>334</v>
       </c>
@@ -5216,7 +5213,7 @@
       <c r="M55" s="17"/>
       <c r="N55" s="3"/>
     </row>
-    <row r="56" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A56" s="19" t="s">
         <v>338</v>
       </c>
@@ -5248,7 +5245,7 @@
       <c r="M56" s="3"/>
       <c r="N56" s="3"/>
     </row>
-    <row r="57" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A57" s="19" t="s">
         <v>344</v>
       </c>
@@ -5280,7 +5277,7 @@
       <c r="M57" s="3"/>
       <c r="N57" s="3"/>
     </row>
-    <row r="58" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="19" t="s">
         <v>351</v>
       </c>
@@ -5312,7 +5309,7 @@
       <c r="M58" s="3"/>
       <c r="N58" s="3"/>
     </row>
-    <row r="59" spans="1:14" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="9" t="s">
         <v>355</v>
       </c>
@@ -5335,15 +5332,15 @@
         <v>361</v>
       </c>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B63" s="28"/>
       <c r="C63" s="28"/>
     </row>
-    <row r="64" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B64" s="29"/>
       <c r="C64" s="30"/>
     </row>
-    <row r="65" spans="2:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:3" ht="16" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B65" s="28"/>
       <c r="C65" s="28"/>
     </row>
@@ -5367,17 +5364,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{273AFAA3-99F7-4E93-9580-DCAE2B14D938}">
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.140625" customWidth="1"/>
-    <col min="2" max="2" width="18.42578125" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" customWidth="1"/>
-    <col min="6" max="6" width="16.42578125" customWidth="1"/>
-    <col min="7" max="7" width="41.42578125" customWidth="1"/>
+    <col min="1" max="1" width="19.1640625" customWidth="1"/>
+    <col min="2" max="2" width="18.5" customWidth="1"/>
+    <col min="4" max="4" width="15.1640625" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" customWidth="1"/>
+    <col min="6" max="6" width="16.5" customWidth="1"/>
+    <col min="7" max="7" width="41.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="195.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="195.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>362</v>
       </c>
@@ -5400,7 +5397,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>364</v>
       </c>
@@ -5432,10 +5429,10 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2489EBC-5098-4697-9724-F190D24E1C3D}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="111" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="111" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>367</v>
       </c>
@@ -5449,13 +5446,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0062C35-A590-498D-8635-16DE3DC0B82A}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="36.42578125" customWidth="1"/>
+    <col min="1" max="1" width="36.5" customWidth="1"/>
     <col min="2" max="2" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>100</v>
       </c>
@@ -5463,7 +5460,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>368</v>
       </c>
@@ -5471,7 +5468,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>370</v>
       </c>
@@ -5487,15 +5484,15 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9E8E4E8-143C-4C64-99FB-1306F2338EFB}">
   <dimension ref="A2:J9"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="27.7109375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="27.42578125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="60.140625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="47.7109375" style="3" customWidth="1"/>
+    <col min="2" max="2" width="27.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="27.5" style="3" customWidth="1"/>
+    <col min="4" max="4" width="60.1640625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="47.6640625" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="B2" s="15" t="s">
         <v>371</v>
       </c>
@@ -5503,7 +5500,7 @@
       <c r="D2" s="12"/>
       <c r="E2" s="12"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="B3" s="16" t="s">
         <v>372</v>
       </c>
@@ -5517,7 +5514,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="156" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="156" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="14" t="s">
         <v>375</v>
       </c>
@@ -5529,7 +5526,7 @@
       </c>
       <c r="E4" s="14"/>
     </row>
-    <row r="5" spans="1:10" ht="182.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="182.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="14" t="s">
         <v>378</v>
       </c>
@@ -5541,7 +5538,7 @@
       </c>
       <c r="E5" s="14"/>
     </row>
-    <row r="6" spans="1:10" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="19"/>
       <c r="B6" s="3" t="s">
         <v>339</v>
@@ -5558,7 +5555,7 @@
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
     </row>
-    <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="B7" s="14" t="s">
         <v>382</v>
       </c>
@@ -5570,7 +5567,7 @@
       </c>
       <c r="E7" s="14"/>
     </row>
-    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="B8" s="14" t="s">
         <v>384</v>
       </c>
@@ -5582,7 +5579,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="90" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="80" x14ac:dyDescent="0.2">
       <c r="B9" s="14"/>
       <c r="C9" s="14" t="s">
         <v>387</v>
@@ -5601,15 +5598,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
@@ -5618,6 +5606,15 @@
     <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5828,14 +5825,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -5848,6 +5837,14 @@
     <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>